<commit_message>
Agregar v2: renders, blend, rentabilidad y gastos actualizados
</commit_message>
<xml_diff>
--- a/entrega-final/Gastos.xlsx
+++ b/entrega-final/Gastos.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Gastos" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,15 +23,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="182">
   <si>
     <t xml:space="preserve">Gastos de la idea final</t>
   </si>
   <si>
     <t xml:space="preserve">Total con IVA en dólares</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Malla sobre cables. Solo la opción elegida de cada ítem. Precios al 1/10/2026.</t>
   </si>
   <si>
     <t xml:space="preserve">Total con IVA en pesos</t>
@@ -578,13 +575,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="&quot;US$ &quot;#,##0.00"/>
     <numFmt numFmtId="166" formatCode="&quot;$ &quot;#,##0"/>
-    <numFmt numFmtId="167" formatCode="&quot;US$ &quot;#,##0.00"/>
-    <numFmt numFmtId="168" formatCode="&quot;$ &quot;#,##0"/>
-    <numFmt numFmtId="169" formatCode="0\ %"/>
+    <numFmt numFmtId="167" formatCode="0\ %"/>
   </numFmts>
   <fonts count="25">
     <font>
@@ -923,260 +918,256 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="63">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="11" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="15" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="15" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="15" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="15" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="21" fillId="7" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="7" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="21" fillId="7" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="7" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1263,9 +1254,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>5123160</xdr:colOff>
+      <xdr:colOff>5122800</xdr:colOff>
       <xdr:row>42</xdr:row>
-      <xdr:rowOff>113040</xdr:rowOff>
+      <xdr:rowOff>112680</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1279,7 +1270,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="5362560"/>
-          <a:ext cx="7237800" cy="4494600"/>
+          <a:ext cx="7237440" cy="4494240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1561,11 +1552,9 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="5"/>
+      <c r="G2" s="3" t="s">
         <v>2</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>3</v>
       </c>
       <c r="H2" s="3"/>
       <c r="I2" s="6" t="n">
@@ -1586,55 +1575,55 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="C4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="D4" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="E4" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="F4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="G4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="H4" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="I4" s="8" t="s">
         <v>11</v>
-      </c>
-      <c r="I4" s="8" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="10" t="s">
         <v>13</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>14</v>
       </c>
       <c r="C5" s="11" t="n">
         <f aca="false">1</f>
         <v>1</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E5" s="12" t="n">
         <v>14650</v>
       </c>
       <c r="F5" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="14" t="s">
         <v>16</v>
-      </c>
-      <c r="G5" s="14" t="s">
-        <v>17</v>
       </c>
       <c r="H5" s="15" t="n">
         <f aca="false">C5*E5</f>
@@ -1647,26 +1636,26 @@
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>18</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>19</v>
       </c>
       <c r="C6" s="11" t="n">
         <f aca="false">Supuestos!$B$6/3*Supuestos!$B$8+Supuestos!$B$9</f>
         <v>18</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E6" s="12" t="n">
         <v>112.29</v>
       </c>
       <c r="F6" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" s="14" t="s">
         <v>16</v>
-      </c>
-      <c r="G6" s="14" t="s">
-        <v>17</v>
       </c>
       <c r="H6" s="15" t="n">
         <f aca="false">C6*E6</f>
@@ -1679,26 +1668,26 @@
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C7" s="11" t="n">
         <f aca="false">ROUNDUP(Supuestos!$B$6/INT(6/Supuestos!$B$10),0)</f>
         <v>3</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E7" s="12" t="n">
         <v>312.14</v>
       </c>
       <c r="F7" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="14" t="s">
         <v>16</v>
-      </c>
-      <c r="G7" s="14" t="s">
-        <v>17</v>
       </c>
       <c r="H7" s="15" t="n">
         <f aca="false">C7*E7</f>
@@ -1711,26 +1700,26 @@
     </row>
     <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C8" s="11" t="n">
         <f aca="false">ROUNDUP(Supuestos!$B$6*Supuestos!$B$11/6,0)</f>
         <v>2</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E8" s="12" t="n">
         <v>94.11</v>
       </c>
       <c r="F8" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G8" s="14" t="s">
         <v>16</v>
-      </c>
-      <c r="G8" s="14" t="s">
-        <v>17</v>
       </c>
       <c r="H8" s="15" t="n">
         <f aca="false">C8*E8</f>
@@ -1743,26 +1732,26 @@
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C9" s="11" t="n">
         <f aca="false">1</f>
         <v>1</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E9" s="12" t="n">
         <v>140.81</v>
       </c>
       <c r="F9" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" s="14" t="s">
         <v>16</v>
-      </c>
-      <c r="G9" s="14" t="s">
-        <v>17</v>
       </c>
       <c r="H9" s="15" t="n">
         <f aca="false">C9*E9</f>
@@ -1775,26 +1764,26 @@
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C10" s="11" t="n">
         <f aca="false">ROUNDUP((Supuestos!$B$12*Supuestos!$B$13+Supuestos!$B$6*Supuestos!$B$14)/6,0)</f>
         <v>1</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E10" s="12" t="n">
         <v>140.07</v>
       </c>
       <c r="F10" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G10" s="14" t="s">
         <v>16</v>
-      </c>
-      <c r="G10" s="14" t="s">
-        <v>17</v>
       </c>
       <c r="H10" s="15" t="n">
         <f aca="false">C10*E10</f>
@@ -1807,26 +1796,26 @@
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="18" t="s">
         <v>26</v>
-      </c>
-      <c r="B11" s="18" t="s">
-        <v>27</v>
       </c>
       <c r="C11" s="19" t="n">
         <f aca="false">Supuestos!$B$15*Supuestos!$B$16</f>
         <v>215</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E11" s="20" t="n">
         <v>495</v>
       </c>
       <c r="F11" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="G11" s="22" t="s">
         <v>29</v>
-      </c>
-      <c r="G11" s="22" t="s">
-        <v>30</v>
       </c>
       <c r="H11" s="23" t="n">
         <f aca="false">C11*E11</f>
@@ -1839,26 +1828,26 @@
     </row>
     <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C12" s="19" t="n">
         <f aca="false">Supuestos!$B$17*Supuestos!$B$18</f>
         <v>27</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E12" s="20" t="n">
         <v>285</v>
       </c>
       <c r="F12" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="G12" s="22" t="s">
         <v>29</v>
-      </c>
-      <c r="G12" s="22" t="s">
-        <v>30</v>
       </c>
       <c r="H12" s="23" t="n">
         <f aca="false">C12*E12</f>
@@ -1871,26 +1860,26 @@
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C13" s="11" t="n">
         <f aca="false">Supuestos!$B$15*2</f>
         <v>10</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E13" s="12" t="n">
         <v>40.43</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H13" s="15" t="n">
         <f aca="false">C13*E13</f>
@@ -1903,26 +1892,26 @@
     </row>
     <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C14" s="11" t="n">
         <f aca="false">Supuestos!$B$17*2</f>
         <v>6</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E14" s="12" t="n">
         <v>16.58</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H14" s="15" t="n">
         <f aca="false">C14*E14</f>
@@ -1935,26 +1924,26 @@
     </row>
     <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C15" s="19" t="n">
         <f aca="false">Supuestos!$B$15</f>
         <v>5</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E15" s="20" t="n">
         <v>1165</v>
       </c>
       <c r="F15" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="G15" s="22" t="s">
         <v>29</v>
-      </c>
-      <c r="G15" s="22" t="s">
-        <v>30</v>
       </c>
       <c r="H15" s="23" t="n">
         <f aca="false">C15*E15</f>
@@ -1967,26 +1956,26 @@
     </row>
     <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="17" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C16" s="19" t="n">
         <f aca="false">Supuestos!$B$17</f>
         <v>3</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E16" s="20" t="n">
         <v>506</v>
       </c>
       <c r="F16" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="G16" s="22" t="s">
         <v>29</v>
-      </c>
-      <c r="G16" s="22" t="s">
-        <v>30</v>
       </c>
       <c r="H16" s="23" t="n">
         <f aca="false">C16*E16</f>
@@ -1999,26 +1988,26 @@
     </row>
     <row r="17" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C17" s="19" t="n">
         <f aca="false">Supuestos!$B$15*2*Supuestos!$B$19</f>
         <v>30</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E17" s="20" t="n">
         <v>137</v>
       </c>
       <c r="F17" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="G17" s="22" t="s">
         <v>29</v>
-      </c>
-      <c r="G17" s="22" t="s">
-        <v>30</v>
       </c>
       <c r="H17" s="23" t="n">
         <f aca="false">C17*E17</f>
@@ -2031,26 +2020,26 @@
     </row>
     <row r="18" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="17" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C18" s="19" t="n">
         <f aca="false">Supuestos!$B$17*2*Supuestos!$B$19</f>
         <v>18</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E18" s="20" t="n">
         <v>96</v>
       </c>
       <c r="F18" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="G18" s="22" t="s">
         <v>29</v>
-      </c>
-      <c r="G18" s="22" t="s">
-        <v>30</v>
       </c>
       <c r="H18" s="23" t="n">
         <f aca="false">C18*E18</f>
@@ -2063,26 +2052,26 @@
     </row>
     <row r="19" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" s="18" t="s">
         <v>39</v>
-      </c>
-      <c r="B19" s="18" t="s">
-        <v>40</v>
       </c>
       <c r="C19" s="19" t="n">
         <f aca="false">ROUNDUP(Supuestos!$B$12*Supuestos!$B$20/Supuestos!$B$21,0)</f>
         <v>4</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E19" s="20" t="n">
         <v>1696</v>
       </c>
       <c r="F19" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="G19" s="22" t="s">
         <v>29</v>
-      </c>
-      <c r="G19" s="22" t="s">
-        <v>30</v>
       </c>
       <c r="H19" s="23" t="n">
         <f aca="false">C19*E19</f>
@@ -2095,26 +2084,26 @@
     </row>
     <row r="20" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C20" s="19" t="n">
         <f aca="false">ROUNDUP(Supuestos!$B$12*Supuestos!$B$20*Supuestos!$B$22,0)+ROUNDUP(Supuestos!$B$6/Supuestos!$B$23,0)</f>
         <v>14</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E20" s="20" t="n">
         <v>169</v>
       </c>
       <c r="F20" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="G20" s="22" t="s">
         <v>29</v>
-      </c>
-      <c r="G20" s="22" t="s">
-        <v>30</v>
       </c>
       <c r="H20" s="23" t="n">
         <f aca="false">C20*E20</f>
@@ -2127,26 +2116,26 @@
     </row>
     <row r="21" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C21" s="19" t="n">
         <f aca="false">ROUNDUP((Supuestos!$B$12*Supuestos!$B$20+Supuestos!$B$6*2)/20,0)</f>
         <v>4</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E21" s="20" t="n">
         <v>249</v>
       </c>
       <c r="F21" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="G21" s="22" t="s">
         <v>29</v>
-      </c>
-      <c r="G21" s="22" t="s">
-        <v>30</v>
       </c>
       <c r="H21" s="23" t="n">
         <f aca="false">C21*E21</f>
@@ -2159,26 +2148,26 @@
     </row>
     <row r="22" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22" s="18" t="s">
         <v>44</v>
-      </c>
-      <c r="B22" s="18" t="s">
-        <v>45</v>
       </c>
       <c r="C22" s="19" t="n">
         <f aca="false">ROUNDUP(Supuestos!$B$24*Supuestos!$B$25/100,0)</f>
         <v>6</v>
       </c>
       <c r="D22" s="19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E22" s="20" t="n">
         <v>2400</v>
       </c>
       <c r="F22" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="G22" s="22" t="s">
         <v>29</v>
-      </c>
-      <c r="G22" s="22" t="s">
-        <v>30</v>
       </c>
       <c r="H22" s="23" t="n">
         <f aca="false">C22*E22</f>
@@ -2191,14 +2180,14 @@
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="25" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="26"/>
       <c r="D24" s="26"/>
       <c r="E24" s="26"/>
       <c r="F24" s="27" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G24" s="26"/>
       <c r="H24" s="28" t="n">
@@ -2212,14 +2201,14 @@
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="25" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="26"/>
       <c r="D25" s="26"/>
       <c r="E25" s="26"/>
       <c r="F25" s="27" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G25" s="26"/>
       <c r="H25" s="29" t="n">
@@ -2233,7 +2222,7 @@
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="30" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B27" s="30"/>
       <c r="C27" s="30"/>
@@ -2246,7 +2235,7 @@
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="31" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B28" s="31"/>
       <c r="C28" s="31"/>
@@ -2259,7 +2248,7 @@
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B29" s="31"/>
       <c r="C29" s="31"/>
@@ -2308,12 +2297,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2328,42 +2317,42 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="D4" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="E4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="D4" s="8" t="s">
+      <c r="F4" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="E4" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="F4" s="8" t="s">
+      <c r="G4" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="H4" s="8" t="s">
         <v>58</v>
-      </c>
-      <c r="H4" s="8" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="18" t="s">
         <v>13</v>
-      </c>
-      <c r="B5" s="18" t="s">
-        <v>14</v>
       </c>
       <c r="C5" s="33" t="n">
         <v>14650</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E5" s="19" t="n">
         <f aca="false">1</f>
@@ -2374,24 +2363,24 @@
         <v>14650</v>
       </c>
       <c r="G5" s="35" t="s">
+        <v>59</v>
+      </c>
+      <c r="H5" s="36" t="s">
         <v>60</v>
-      </c>
-      <c r="H5" s="36" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="38" t="s">
         <v>18</v>
-      </c>
-      <c r="B6" s="38" t="s">
-        <v>19</v>
       </c>
       <c r="C6" s="39" t="n">
         <v>112.29</v>
       </c>
       <c r="D6" s="40" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E6" s="41" t="n">
         <f aca="false">Supuestos!$B$6/3*Supuestos!$B$8+Supuestos!$B$9</f>
@@ -2402,24 +2391,24 @@
         <v>2021.22</v>
       </c>
       <c r="G6" s="43" t="s">
+        <v>61</v>
+      </c>
+      <c r="H6" s="44" t="s">
         <v>62</v>
-      </c>
-      <c r="H6" s="44" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C7" s="33" t="n">
         <v>312.14</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E7" s="19" t="n">
         <f aca="false">ROUNDUP(Supuestos!$B$6/INT(6/Supuestos!$B$10),0)</f>
@@ -2430,24 +2419,24 @@
         <v>936.42</v>
       </c>
       <c r="G7" s="35" t="s">
+        <v>63</v>
+      </c>
+      <c r="H7" s="36" t="s">
         <v>64</v>
-      </c>
-      <c r="H7" s="36" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="37" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C8" s="39" t="n">
         <v>94.11</v>
       </c>
       <c r="D8" s="40" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E8" s="41" t="n">
         <f aca="false">ROUNDUP(Supuestos!$B$6*Supuestos!$B$11/6,0)</f>
@@ -2458,24 +2447,24 @@
         <v>188.22</v>
       </c>
       <c r="G8" s="43" t="s">
+        <v>65</v>
+      </c>
+      <c r="H8" s="44" t="s">
         <v>66</v>
-      </c>
-      <c r="H8" s="44" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C9" s="33" t="n">
         <v>140.07</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E9" s="19" t="n">
         <f aca="false">ROUNDUP((Supuestos!$B$12*Supuestos!$B$13+Supuestos!$B$6*Supuestos!$B$14)/6,0)</f>
@@ -2486,24 +2475,24 @@
         <v>140.07</v>
       </c>
       <c r="G9" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="H9" s="36" t="s">
         <v>68</v>
-      </c>
-      <c r="H9" s="36" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="37" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="38" t="s">
         <v>26</v>
-      </c>
-      <c r="B10" s="38" t="s">
-        <v>27</v>
       </c>
       <c r="C10" s="45" t="n">
         <v>495</v>
       </c>
       <c r="D10" s="40" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E10" s="41" t="n">
         <f aca="false">Supuestos!$B$15*Supuestos!$B$16</f>
@@ -2514,24 +2503,24 @@
         <v>106425</v>
       </c>
       <c r="G10" s="43" t="s">
+        <v>69</v>
+      </c>
+      <c r="H10" s="44" t="s">
         <v>70</v>
-      </c>
-      <c r="H10" s="44" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>285</v>
       </c>
       <c r="D11" s="22" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E11" s="19" t="n">
         <f aca="false">Supuestos!$B$17*Supuestos!$B$18</f>
@@ -2542,24 +2531,24 @@
         <v>7695</v>
       </c>
       <c r="G11" s="35" t="s">
+        <v>71</v>
+      </c>
+      <c r="H11" s="36" t="s">
         <v>72</v>
-      </c>
-      <c r="H11" s="36" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="37" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B12" s="38" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C12" s="39" t="n">
         <v>40.43</v>
       </c>
       <c r="D12" s="40" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E12" s="41" t="n">
         <f aca="false">Supuestos!$B$15*2</f>
@@ -2570,24 +2559,24 @@
         <v>404.3</v>
       </c>
       <c r="G12" s="43" t="s">
+        <v>73</v>
+      </c>
+      <c r="H12" s="44" t="s">
         <v>74</v>
-      </c>
-      <c r="H12" s="44" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C13" s="33" t="n">
         <v>16.58</v>
       </c>
       <c r="D13" s="22" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E13" s="19" t="n">
         <f aca="false">Supuestos!$B$17*2</f>
@@ -2598,24 +2587,24 @@
         <v>99.48</v>
       </c>
       <c r="G13" s="35" t="s">
+        <v>75</v>
+      </c>
+      <c r="H13" s="36" t="s">
         <v>76</v>
-      </c>
-      <c r="H13" s="36" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="37" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B14" s="38" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C14" s="45" t="n">
         <v>1165</v>
       </c>
       <c r="D14" s="40" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E14" s="41" t="n">
         <f aca="false">Supuestos!$B$15</f>
@@ -2626,24 +2615,24 @@
         <v>5825</v>
       </c>
       <c r="G14" s="43" t="s">
+        <v>77</v>
+      </c>
+      <c r="H14" s="44" t="s">
         <v>78</v>
-      </c>
-      <c r="H14" s="44" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C15" s="23" t="n">
         <v>506</v>
       </c>
       <c r="D15" s="22" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E15" s="19" t="n">
         <f aca="false">Supuestos!$B$17</f>
@@ -2654,24 +2643,24 @@
         <v>1518</v>
       </c>
       <c r="G15" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="H15" s="36" t="s">
         <v>80</v>
-      </c>
-      <c r="H15" s="36" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="37" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B16" s="38" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C16" s="45" t="n">
         <v>137</v>
       </c>
       <c r="D16" s="40" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E16" s="41" t="n">
         <f aca="false">Supuestos!$B$15*2*Supuestos!$B$19</f>
@@ -2682,24 +2671,24 @@
         <v>4110</v>
       </c>
       <c r="G16" s="43" t="s">
+        <v>81</v>
+      </c>
+      <c r="H16" s="44" t="s">
         <v>82</v>
-      </c>
-      <c r="H16" s="44" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>96</v>
       </c>
       <c r="D17" s="22" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E17" s="19" t="n">
         <f aca="false">Supuestos!$B$17*2*Supuestos!$B$19</f>
@@ -2710,24 +2699,24 @@
         <v>1728</v>
       </c>
       <c r="G17" s="35" t="s">
+        <v>83</v>
+      </c>
+      <c r="H17" s="36" t="s">
         <v>84</v>
-      </c>
-      <c r="H17" s="36" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="37" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" s="38" t="s">
         <v>39</v>
-      </c>
-      <c r="B18" s="38" t="s">
-        <v>40</v>
       </c>
       <c r="C18" s="45" t="n">
         <v>1696</v>
       </c>
       <c r="D18" s="40" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E18" s="41" t="n">
         <f aca="false">ROUNDUP(Supuestos!$B$12*Supuestos!$B$20/Supuestos!$B$21,0)</f>
@@ -2738,24 +2727,24 @@
         <v>6784</v>
       </c>
       <c r="G18" s="43" t="s">
+        <v>85</v>
+      </c>
+      <c r="H18" s="44" t="s">
         <v>86</v>
-      </c>
-      <c r="H18" s="44" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C19" s="23" t="n">
         <v>169</v>
       </c>
       <c r="D19" s="22" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E19" s="19" t="n">
         <f aca="false">ROUNDUP(Supuestos!$B$12*Supuestos!$B$20*Supuestos!$B$22,0)+ROUNDUP(Supuestos!$B$6/Supuestos!$B$23,0)</f>
@@ -2766,24 +2755,24 @@
         <v>2366</v>
       </c>
       <c r="G19" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="H19" s="36" t="s">
         <v>88</v>
-      </c>
-      <c r="H19" s="36" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="37" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B20" s="38" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C20" s="45" t="n">
         <v>249</v>
       </c>
       <c r="D20" s="40" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E20" s="41" t="n">
         <f aca="false">ROUNDUP((Supuestos!$B$12*Supuestos!$B$20+Supuestos!$B$6*2)/20,0)</f>
@@ -2794,24 +2783,24 @@
         <v>996</v>
       </c>
       <c r="G20" s="43" t="s">
+        <v>89</v>
+      </c>
+      <c r="H20" s="44" t="s">
         <v>90</v>
-      </c>
-      <c r="H20" s="44" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="B21" s="18" t="s">
         <v>44</v>
-      </c>
-      <c r="B21" s="18" t="s">
-        <v>45</v>
       </c>
       <c r="C21" s="23" t="n">
         <v>2400</v>
       </c>
       <c r="D21" s="22" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E21" s="19" t="n">
         <f aca="false">ROUNDUP(Supuestos!$B$24*Supuestos!$B$25/100,0)</f>
@@ -2822,10 +2811,10 @@
         <v>14400</v>
       </c>
       <c r="G21" s="35" t="s">
+        <v>91</v>
+      </c>
+      <c r="H21" s="36" t="s">
         <v>92</v>
-      </c>
-      <c r="H21" s="36" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2840,7 +2829,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="50" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B23" s="50"/>
       <c r="C23" s="50"/>
@@ -2921,7 +2910,7 @@
       <c r="H30" s="52"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="53"/>
+      <c r="A31" s="52"/>
       <c r="B31" s="52"/>
       <c r="C31" s="52"/>
       <c r="D31" s="52"/>
@@ -2979,12 +2968,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2995,410 +2984,410 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B4" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="C4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="8" t="s">
         <v>98</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="B5" s="53" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="C5" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="B5" s="54" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="C5" s="19" t="s">
+      <c r="D5" s="54" t="s">
         <v>101</v>
-      </c>
-      <c r="D5" s="55" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="38" t="s">
+        <v>102</v>
+      </c>
+      <c r="B6" s="55" t="n">
+        <v>12</v>
+      </c>
+      <c r="C6" s="41" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="56" t="s">
         <v>103</v>
-      </c>
-      <c r="B6" s="56" t="n">
-        <v>12</v>
-      </c>
-      <c r="C6" s="41" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6" s="57" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="B7" s="55" t="n">
+        <v>8</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="54" t="s">
         <v>105</v>
-      </c>
-      <c r="B7" s="56" t="n">
-        <v>8</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" s="55" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="38" t="s">
+        <v>106</v>
+      </c>
+      <c r="B8" s="55" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" s="41" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="56" t="s">
         <v>107</v>
-      </c>
-      <c r="B8" s="56" t="n">
-        <v>4</v>
-      </c>
-      <c r="C8" s="41" t="s">
-        <v>33</v>
-      </c>
-      <c r="D8" s="57" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="B9" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="54" t="s">
         <v>109</v>
-      </c>
-      <c r="B9" s="56" t="n">
-        <v>2</v>
-      </c>
-      <c r="C9" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9" s="55" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="38" t="s">
+        <v>110</v>
+      </c>
+      <c r="B10" s="55" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="C10" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="56" t="s">
         <v>111</v>
-      </c>
-      <c r="B10" s="56" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="C10" s="41" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="57" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="B11" s="55" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="54" t="s">
         <v>113</v>
-      </c>
-      <c r="B11" s="56" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" s="55" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="38" t="s">
+        <v>114</v>
+      </c>
+      <c r="B12" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="C12" s="41" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="56" t="s">
         <v>115</v>
-      </c>
-      <c r="B12" s="56" t="n">
-        <v>10</v>
-      </c>
-      <c r="C12" s="41" t="s">
-        <v>33</v>
-      </c>
-      <c r="D12" s="57" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="B13" s="55" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="54" t="s">
         <v>117</v>
-      </c>
-      <c r="B13" s="56" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C13" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="D13" s="55" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="38" t="s">
+        <v>118</v>
+      </c>
+      <c r="B14" s="55" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C14" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="56" t="s">
         <v>119</v>
-      </c>
-      <c r="B14" s="56" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C14" s="41" t="s">
-        <v>28</v>
-      </c>
-      <c r="D14" s="57" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="B15" s="55" t="n">
+        <v>5</v>
+      </c>
+      <c r="C15" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="D15" s="54" t="s">
         <v>121</v>
-      </c>
-      <c r="B15" s="56" t="n">
-        <v>5</v>
-      </c>
-      <c r="C15" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="D15" s="55" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="38" t="s">
+        <v>122</v>
+      </c>
+      <c r="B16" s="55" t="n">
+        <v>43</v>
+      </c>
+      <c r="C16" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="56" t="s">
         <v>123</v>
-      </c>
-      <c r="B16" s="56" t="n">
-        <v>43</v>
-      </c>
-      <c r="C16" s="41" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="57" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="B17" s="55" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="D17" s="54" t="s">
         <v>125</v>
-      </c>
-      <c r="B17" s="56" t="n">
-        <v>3</v>
-      </c>
-      <c r="C17" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="D17" s="55" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="38" t="s">
+        <v>126</v>
+      </c>
+      <c r="B18" s="55" t="n">
+        <v>9</v>
+      </c>
+      <c r="C18" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="D18" s="56" t="s">
         <v>127</v>
-      </c>
-      <c r="B18" s="56" t="n">
-        <v>9</v>
-      </c>
-      <c r="C18" s="41" t="s">
-        <v>28</v>
-      </c>
-      <c r="D18" s="57" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="B19" s="55" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" s="54" t="s">
         <v>129</v>
-      </c>
-      <c r="B19" s="56" t="n">
-        <v>3</v>
-      </c>
-      <c r="C19" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="D19" s="55" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="B20" s="55" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" s="41" t="s">
+        <v>32</v>
+      </c>
+      <c r="D20" s="56" t="s">
         <v>131</v>
-      </c>
-      <c r="B20" s="56" t="n">
-        <v>4</v>
-      </c>
-      <c r="C20" s="41" t="s">
-        <v>33</v>
-      </c>
-      <c r="D20" s="57" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="B21" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="C21" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="D21" s="54" t="s">
         <v>133</v>
-      </c>
-      <c r="B21" s="56" t="n">
-        <v>10</v>
-      </c>
-      <c r="C21" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="D21" s="55" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="38" t="s">
+        <v>134</v>
+      </c>
+      <c r="B22" s="55" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C22" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="D22" s="56" t="s">
         <v>135</v>
-      </c>
-      <c r="B22" s="56" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="C22" s="41" t="s">
-        <v>28</v>
-      </c>
-      <c r="D22" s="57" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
+        <v>136</v>
+      </c>
+      <c r="B23" s="55" t="n">
+        <v>3</v>
+      </c>
+      <c r="C23" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="D23" s="54" t="s">
         <v>137</v>
-      </c>
-      <c r="B23" s="56" t="n">
-        <v>3</v>
-      </c>
-      <c r="C23" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="D23" s="55" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="38" t="s">
+        <v>138</v>
+      </c>
+      <c r="B24" s="55" t="n">
+        <v>508</v>
+      </c>
+      <c r="C24" s="41" t="s">
+        <v>32</v>
+      </c>
+      <c r="D24" s="56" t="s">
         <v>139</v>
-      </c>
-      <c r="B24" s="56" t="n">
-        <v>508</v>
-      </c>
-      <c r="C24" s="41" t="s">
-        <v>33</v>
-      </c>
-      <c r="D24" s="57" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="B25" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D25" s="54" t="s">
         <v>141</v>
-      </c>
-      <c r="B25" s="56" t="n">
-        <v>1</v>
-      </c>
-      <c r="C25" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="D25" s="55" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="38" t="s">
-        <v>143</v>
-      </c>
-      <c r="B26" s="56" t="n">
+        <v>142</v>
+      </c>
+      <c r="B26" s="55" t="n">
         <f aca="false">41*24.5</f>
         <v>1004.5</v>
       </c>
       <c r="C26" s="41" t="s">
+        <v>143</v>
+      </c>
+      <c r="D26" s="56" t="s">
         <v>144</v>
-      </c>
-      <c r="D26" s="57" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
-        <v>146</v>
-      </c>
-      <c r="B27" s="56" t="n">
+        <v>145</v>
+      </c>
+      <c r="B27" s="55" t="n">
         <f aca="false">1*4.2</f>
         <v>4.2</v>
       </c>
       <c r="C27" s="19" t="s">
-        <v>144</v>
-      </c>
-      <c r="D27" s="55" t="s">
+        <v>143</v>
+      </c>
+      <c r="D27" s="54" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="57" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="58" t="s">
+    <row r="30" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="58" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="30" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="59" t="s">
+      <c r="B30" s="58"/>
+      <c r="C30" s="58"/>
+      <c r="D30" s="58"/>
+    </row>
+    <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="58" t="s">
         <v>149</v>
       </c>
-      <c r="B30" s="59"/>
-      <c r="C30" s="59"/>
-      <c r="D30" s="59"/>
-    </row>
-    <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="59" t="s">
+      <c r="B31" s="58"/>
+      <c r="C31" s="58"/>
+      <c r="D31" s="58"/>
+    </row>
+    <row r="32" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="58" t="s">
         <v>150</v>
       </c>
-      <c r="B31" s="59"/>
-      <c r="C31" s="59"/>
-      <c r="D31" s="59"/>
-    </row>
-    <row r="32" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="59" t="s">
+      <c r="B32" s="58"/>
+      <c r="C32" s="58"/>
+      <c r="D32" s="58"/>
+    </row>
+    <row r="33" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="58" t="s">
         <v>151</v>
       </c>
-      <c r="B32" s="59"/>
-      <c r="C32" s="59"/>
-      <c r="D32" s="59"/>
-    </row>
-    <row r="33" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="59" t="s">
+      <c r="B33" s="58"/>
+      <c r="C33" s="58"/>
+      <c r="D33" s="58"/>
+    </row>
+    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="58" t="s">
         <v>152</v>
       </c>
-      <c r="B33" s="59"/>
-      <c r="C33" s="59"/>
-      <c r="D33" s="59"/>
-    </row>
-    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="59" t="s">
+      <c r="B34" s="58"/>
+      <c r="C34" s="58"/>
+      <c r="D34" s="58"/>
+    </row>
+    <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="58" t="s">
         <v>153</v>
       </c>
-      <c r="B34" s="59"/>
-      <c r="C34" s="59"/>
-      <c r="D34" s="59"/>
-    </row>
-    <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="59" t="s">
+      <c r="B35" s="58"/>
+      <c r="C35" s="58"/>
+      <c r="D35" s="58"/>
+    </row>
+    <row r="36" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="58" t="s">
         <v>154</v>
       </c>
-      <c r="B35" s="59"/>
-      <c r="C35" s="59"/>
-      <c r="D35" s="59"/>
-    </row>
-    <row r="36" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="59" t="s">
+      <c r="B36" s="58"/>
+      <c r="C36" s="58"/>
+      <c r="D36" s="58"/>
+    </row>
+    <row r="37" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="58" t="s">
         <v>155</v>
       </c>
-      <c r="B36" s="59"/>
-      <c r="C36" s="59"/>
-      <c r="D36" s="59"/>
-    </row>
-    <row r="37" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="59" t="s">
-        <v>156</v>
-      </c>
-      <c r="B37" s="59"/>
-      <c r="C37" s="59"/>
-      <c r="D37" s="59"/>
+      <c r="B37" s="58"/>
+      <c r="C37" s="58"/>
+      <c r="D37" s="58"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -3436,12 +3425,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3449,108 +3438,108 @@
       <c r="B3" s="7"/>
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="60" t="s">
+      <c r="A4" s="59" t="s">
+        <v>158</v>
+      </c>
+      <c r="B4" s="60"/>
+    </row>
+    <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="61" t="s">
         <v>159</v>
       </c>
-      <c r="B4" s="61"/>
-    </row>
-    <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="62" t="s">
+      <c r="B5" s="18" t="s">
         <v>160</v>
       </c>
-      <c r="B5" s="18" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="61" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="62" t="s">
+      <c r="B6" s="18" t="s">
         <v>162</v>
       </c>
-      <c r="B6" s="18" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="61" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="62" t="s">
+      <c r="B7" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="B7" s="18" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="61" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="62" t="s">
+      <c r="B8" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="B8" s="18" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="61" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="62" t="s">
+      <c r="B9" s="18" t="s">
         <v>168</v>
       </c>
-      <c r="B9" s="18" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="61" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="62" t="s">
+      <c r="B10" s="18" t="s">
         <v>170</v>
       </c>
-      <c r="B10" s="18" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="59" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="60" t="s">
+      <c r="B12" s="60"/>
+    </row>
+    <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="61" t="s">
         <v>172</v>
       </c>
-      <c r="B12" s="61"/>
-    </row>
-    <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="62" t="s">
+      <c r="B13" s="18" t="s">
         <v>173</v>
       </c>
-      <c r="B13" s="18" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="61" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="62" t="s">
+      <c r="B14" s="18" t="s">
         <v>175</v>
       </c>
-      <c r="B14" s="18" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="61" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="62" t="s">
+      <c r="B15" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="B15" s="18" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="61" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="62" t="s">
+      <c r="B16" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="B16" s="18" t="s">
+    </row>
+    <row r="18" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="59" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="60" t="s">
+      <c r="B18" s="60"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="62" t="s">
         <v>181</v>
       </c>
-      <c r="B18" s="61"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="63" t="s">
-        <v>182</v>
-      </c>
-      <c r="B19" s="63"/>
+      <c r="B19" s="62"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>